<commit_message>
Change Note to Supplemental Guidance
to match what the components declares there. This is to help make updating this section less confusing by making it clear what goes to what.
</commit_message>
<xml_diff>
--- a/assessments/FinOps Foundation/assessment.xlsx
+++ b/assessments/FinOps Foundation/assessment.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="385">
   <si>
     <t>Sum of Weights</t>
   </si>
@@ -956,6 +956,26 @@
   </si>
   <si>
     <t>022</t>
+  </si>
+  <si>
+    <t>* Select which teams or groups are in scope for the planned assessments
+* Select which capabilities/actions are in scope for each group's assessment
+* Select weights for each included action based on goals of the assessment and importance to the business
+* Set a preliminary target score for each included action to use for comparison
+10*Ceil(x/4)</t>
+  </si>
+  <si>
+    <t>* Use objective (not subjective) scoring metrics for assessment evaluation
+* Document how metrics used in the assessment are calculated and state all assumptions
+* Use the same calculation assumptions and formulas across scopes if possible
+* List relevant documentation of process and policy as evidentiary support for each score
+10*Ceil(x/4)</t>
+  </si>
+  <si>
+    <t>* Complete an initial assessment for different scopes of the business to establish a baseline
+* Plot scores over time to track maturity progress for priority scopes
+* Complete analysis on what contributed to or hindered progress across scopes or different areas of the assessment
+10*Ceil(x/3)</t>
   </si>
   <si>
     <t>* Define process for reviewing asking for credits from CSPs
@@ -1010,10 +1030,45 @@
 10*Ceil(x/4)</t>
   </si>
   <si>
+    <t>* Defined scope of each project to be estimated
+* Developed list of known inputs to the project
+* Have a process to determine what may be missing from the inputs or scope
+* Have a policy review to determine additional needs for inputs or scope
+* For each component of the estimate, list all assumptions
+10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Inventory possible commitment based discounts (RIs, Savings Plans, CUDs, etc.) available for deployed resources
+* Consider any private negotiated line item discounts vs public RI/CUD discounts
+* Set resource type standards to make use of spend commitments while maintaining needs of the business
+* Scenario plan commitment options versus potential changes in resources
+* Reference commit allocation strategy to calculate cost impact of shared scope vs private account commitments
+10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Use pricing lists or pricing calculators to estimate workload spend
+* Run workloads as trial experiments to get baseline spend
+* Estimate workload costs based on similar applications already deployed in your environment
+* Determine fixed costs vs formulas for variable costs due to growth of workloads
+* Factor in discounts and uptime metrics to determine accurate spend vs list
+10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>1. Calculate kg of carbon dioxide equivalents (kgCO2e), or similar, for new and ongoing workloads
+2. Compare carbon calculations with targets for new projects and overall consumption</t>
+  </si>
+  <si>
     <t>* Define and follow process for gathering deployment plans from teams
 * Determine timeline for each new project to adjust the forecast during that time
 * Determine how optimizations and lower run rate will impact the forecast on a rolling basis
 10*Ceil(x/3)</t>
+  </si>
+  <si>
+    <t>* Refer teams to Documented Estimating Scope &amp; Policy and include these methods in trainings
+* Teams track baseline spend for resources they own, and share changes to baseline with leadership
+* Teams will share updates about their change in usage of shared resources and dependencies
+* Track team adoption of better estimates via KPIs around baseline or plan vs actuals
+10*Ceil(x/4)</t>
   </si>
   <si>
     <t>* Define cost drivers from finance/business
@@ -1126,6 +1181,15 @@
     <t>[{'Score': 0, 'Condition': 'Not monitored'}, {'Score': 2, 'Condition': 'Reported'}, {'Score': 5, 'Condition': 'Manual remediation'}, {'Score': 10, 'Condition': 'Automated remediation'}]</t>
   </si>
   <si>
+    <t>[{'Score': 0, 'Condition': '0 items completed'}, {'Score': 3, 'Condition': '1 item completed'}, {'Score': 5, 'Condition': '2 items completed'}, {'Score': 8, 'Condition': '3 items completed'}, {'Score': 10, 'Condition': '4 items completed'}]</t>
+  </si>
+  <si>
+    <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 3, 'Condition': '1 item completed'}, {'Score': 5, 'Condition': '2 items completed'}, {'Score': 8, 'Condition': '3 items completed'}, {'Score': 10, 'Condition': '4 items completed'}]</t>
+  </si>
+  <si>
+    <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 4, 'Condition': '1 item completed'}, {'Score': 7, 'Condition': '2 items completed'}, {'Score': 10, 'Condition': '3 items completed'}]</t>
+  </si>
+  <si>
     <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 5, 'Condition': '1 item completed'}, {'Score': 10, 'Condition': '2 items completed'}]</t>
   </si>
   <si>
@@ -1141,9 +1205,6 @@
     <t>[{'Score': 0, 'Condition': 'Not done'}, {'Score': 10, 'Condition': 'Done and clearly defined'}]</t>
   </si>
   <si>
-    <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 4, 'Condition': '1 item completed'}, {'Score': 7, 'Condition': '2 items completed'}, {'Score': 10, 'Condition': '3 items completed'}]</t>
-  </si>
-  <si>
     <t>[{'Score': 0, 'Condition': 'Does not exist'}, {'Score': 10, 'Condition': 'Exists'}]</t>
   </si>
   <si>
@@ -1162,15 +1223,15 @@
     <t>[{'Score': 0, 'Condition': 'No review of trends'}, {'Score': 3, 'Condition': 'Manual review of trends'}, {'Score': 6, 'Condition': 'Automated trend detection'}, {'Score': 10, 'Condition': 'Manual review and automated trend detection'}]</t>
   </si>
   <si>
-    <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 3, 'Condition': '1 item completed'}, {'Score': 5, 'Condition': '2 items completed'}, {'Score': 8, 'Condition': '3 items completed'}, {'Score': 10, 'Condition': '4 items completed'}]</t>
-  </si>
-  <si>
     <t>[{'Score': 0, 'Condition': 'None'}, {'Score': 1, 'Condition': 'Annual'}, {'Score': 2, 'Condition': 'Quarterly'}, {'Score': 5, 'Condition': 'Monthly'}, {'Score': 7, 'Condition': 'Bi-Weekly'}, {'Score': 8, 'Condition': 'Weekly'}, {'Score': 10, 'Condition': 'Daily'}]</t>
   </si>
   <si>
     <t>[{'Score': 0, 'Condition': 'No alerting'}, {'Score': 10, 'Condition': 'Alerting exists'}]</t>
   </si>
   <si>
+    <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 5, 'Condition': 'item 1 completed'}, {'Score': 10, 'Condition': 'item 2 completed'}]</t>
+  </si>
+  <si>
     <t>[{'Score': 0, 'Condition': 'None'}, {'Score': 10, 'Condition': 'set goal thresholds for kpis and unit costs'}]</t>
   </si>
   <si>
@@ -1199,6 +1260,9 @@
   </si>
   <si>
     <t>0: Not monitored</t>
+  </si>
+  <si>
+    <t>0: 0 items completed</t>
   </si>
   <si>
     <t>0: No items completed</t>
@@ -2569,7 +2633,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H2">
         <f>E2*VALUE(LEFT(G2, FIND(":", G2)-1))</f>
@@ -2595,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H3">
         <f>E3*VALUE(LEFT(G3, FIND(":", G3)-1))</f>
@@ -2621,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H4">
         <f>E4*VALUE(LEFT(G4, FIND(":", G4)-1))</f>
@@ -2647,7 +2711,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
       <c r="H5">
         <f>E5*VALUE(LEFT(G5, FIND(":", G5)-1))</f>
@@ -2673,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H6">
         <f>E6*VALUE(LEFT(G6, FIND(":", G6)-1))</f>
@@ -2698,10 +2762,13 @@
         <v>183</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>313</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="H7">
         <f>E7*VALUE(LEFT(G7, FIND(":", G7)-1))</f>
@@ -2724,10 +2791,13 @@
         <v>184</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>314</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H8">
         <f>E8*VALUE(LEFT(G8, FIND(":", G8)-1))</f>
@@ -2750,10 +2820,13 @@
         <v>185</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>315</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H9">
         <f>E9*VALUE(LEFT(G9, FIND(":", G9)-1))</f>
@@ -2779,7 +2852,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H10">
         <f>E10*VALUE(LEFT(G10, FIND(":", G10)-1))</f>
@@ -2805,7 +2878,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H11">
         <f>E11*VALUE(LEFT(G11, FIND(":", G11)-1))</f>
@@ -2833,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H12">
         <f>E12*VALUE(LEFT(G12, FIND(":", G12)-1))</f>
@@ -2859,7 +2932,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H13">
         <f>E13*VALUE(LEFT(G13, FIND(":", G13)-1))</f>
@@ -2885,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H14">
         <f>E14*VALUE(LEFT(G14, FIND(":", G14)-1))</f>
@@ -2911,10 +2984,10 @@
         <v>1</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H15">
         <f>E15*VALUE(LEFT(G15, FIND(":", G15)-1))</f>
@@ -2940,7 +3013,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H16">
         <f>E16*VALUE(LEFT(G16, FIND(":", G16)-1))</f>
@@ -2968,7 +3041,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H17">
         <f>E17*VALUE(LEFT(G17, FIND(":", G17)-1))</f>
@@ -2994,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H18">
         <f>E18*VALUE(LEFT(G18, FIND(":", G18)-1))</f>
@@ -3020,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H19">
         <f>E19*VALUE(LEFT(G19, FIND(":", G19)-1))</f>
@@ -3046,7 +3119,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H20">
         <f>E20*VALUE(LEFT(G20, FIND(":", G20)-1))</f>
@@ -3072,7 +3145,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H21">
         <f>E21*VALUE(LEFT(G21, FIND(":", G21)-1))</f>
@@ -3098,7 +3171,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H22">
         <f>E22*VALUE(LEFT(G22, FIND(":", G22)-1))</f>
@@ -3126,7 +3199,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H23">
         <f>E23*VALUE(LEFT(G23, FIND(":", G23)-1))</f>
@@ -3152,7 +3225,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="H24">
         <f>E24*VALUE(LEFT(G24, FIND(":", G24)-1))</f>
@@ -3178,7 +3251,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H25">
         <f>E25*VALUE(LEFT(G25, FIND(":", G25)-1))</f>
@@ -3204,10 +3277,10 @@
         <v>1</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H26">
         <f>E26*VALUE(LEFT(G26, FIND(":", G26)-1))</f>
@@ -3233,7 +3306,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H27">
         <f>E27*VALUE(LEFT(G27, FIND(":", G27)-1))</f>
@@ -3261,7 +3334,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H28">
         <f>E28*VALUE(LEFT(G28, FIND(":", G28)-1))</f>
@@ -3287,7 +3360,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H29">
         <f>E29*VALUE(LEFT(G29, FIND(":", G29)-1))</f>
@@ -3313,7 +3386,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H30">
         <f>E30*VALUE(LEFT(G30, FIND(":", G30)-1))</f>
@@ -3339,7 +3412,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H31">
         <f>E31*VALUE(LEFT(G31, FIND(":", G31)-1))</f>
@@ -3365,7 +3438,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H32">
         <f>E32*VALUE(LEFT(G32, FIND(":", G32)-1))</f>
@@ -3391,7 +3464,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H33">
         <f>E33*VALUE(LEFT(G33, FIND(":", G33)-1))</f>
@@ -3419,7 +3492,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H34">
         <f>E34*VALUE(LEFT(G34, FIND(":", G34)-1))</f>
@@ -3445,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H35">
         <f>E35*VALUE(LEFT(G35, FIND(":", G35)-1))</f>
@@ -3471,7 +3544,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H36">
         <f>E36*VALUE(LEFT(G36, FIND(":", G36)-1))</f>
@@ -3497,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H37">
         <f>E37*VALUE(LEFT(G37, FIND(":", G37)-1))</f>
@@ -3523,7 +3596,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H38">
         <f>E38*VALUE(LEFT(G38, FIND(":", G38)-1))</f>
@@ -3549,7 +3622,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H39">
         <f>E39*VALUE(LEFT(G39, FIND(":", G39)-1))</f>
@@ -3577,7 +3650,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H40">
         <f>E40*VALUE(LEFT(G40, FIND(":", G40)-1))</f>
@@ -3603,7 +3676,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H41">
         <f>E41*VALUE(LEFT(G41, FIND(":", G41)-1))</f>
@@ -3629,10 +3702,10 @@
         <v>1</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H42">
         <f>E42*VALUE(LEFT(G42, FIND(":", G42)-1))</f>
@@ -3658,7 +3731,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H43">
         <f>E43*VALUE(LEFT(G43, FIND(":", G43)-1))</f>
@@ -3684,7 +3757,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H44">
         <f>E44*VALUE(LEFT(G44, FIND(":", G44)-1))</f>
@@ -3710,7 +3783,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H45">
         <f>E45*VALUE(LEFT(G45, FIND(":", G45)-1))</f>
@@ -3740,7 +3813,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="H46">
         <f>E46*VALUE(LEFT(G46, FIND(":", G46)-1))</f>
@@ -3766,10 +3839,10 @@
         <v>1</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H47">
         <f>E47*VALUE(LEFT(G47, FIND(":", G47)-1))</f>
@@ -3795,7 +3868,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>367</v>
+        <v>378</v>
       </c>
       <c r="H48">
         <f>E48*VALUE(LEFT(G48, FIND(":", G48)-1))</f>
@@ -3821,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H49">
         <f>E49*VALUE(LEFT(G49, FIND(":", G49)-1))</f>
@@ -3847,7 +3920,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H50">
         <f>E50*VALUE(LEFT(G50, FIND(":", G50)-1))</f>
@@ -3873,7 +3946,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H51">
         <f>E51*VALUE(LEFT(G51, FIND(":", G51)-1))</f>
@@ -3901,7 +3974,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H52">
         <f>E52*VALUE(LEFT(G52, FIND(":", G52)-1))</f>
@@ -3927,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H53">
         <f>E53*VALUE(LEFT(G53, FIND(":", G53)-1))</f>
@@ -3953,7 +4026,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H54">
         <f>E54*VALUE(LEFT(G54, FIND(":", G54)-1))</f>
@@ -3979,7 +4052,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H55">
         <f>E55*VALUE(LEFT(G55, FIND(":", G55)-1))</f>
@@ -4005,7 +4078,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H56">
         <f>E56*VALUE(LEFT(G56, FIND(":", G56)-1))</f>
@@ -4031,7 +4104,7 @@
         <v>0</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H57">
         <f>E57*VALUE(LEFT(G57, FIND(":", G57)-1))</f>
@@ -4059,7 +4132,7 @@
         <v>1</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H58">
         <f>E58*VALUE(LEFT(G58, FIND(":", G58)-1))</f>
@@ -4085,7 +4158,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H59">
         <f>E59*VALUE(LEFT(G59, FIND(":", G59)-1))</f>
@@ -4111,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H60">
         <f>E60*VALUE(LEFT(G60, FIND(":", G60)-1))</f>
@@ -4137,7 +4210,7 @@
         <v>1</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H61">
         <f>E61*VALUE(LEFT(G61, FIND(":", G61)-1))</f>
@@ -4163,7 +4236,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H62">
         <f>E62*VALUE(LEFT(G62, FIND(":", G62)-1))</f>
@@ -4189,7 +4262,7 @@
         <v>0</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H63">
         <f>E63*VALUE(LEFT(G63, FIND(":", G63)-1))</f>
@@ -4217,7 +4290,7 @@
         <v>1</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H64">
         <f>E64*VALUE(LEFT(G64, FIND(":", G64)-1))</f>
@@ -4243,7 +4316,7 @@
         <v>1</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H65">
         <f>E65*VALUE(LEFT(G65, FIND(":", G65)-1))</f>
@@ -4269,7 +4342,7 @@
         <v>0</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H66">
         <f>E66*VALUE(LEFT(G66, FIND(":", G66)-1))</f>
@@ -4295,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H67">
         <f>E67*VALUE(LEFT(G67, FIND(":", G67)-1))</f>
@@ -4321,7 +4394,7 @@
         <v>0</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H68">
         <f>E68*VALUE(LEFT(G68, FIND(":", G68)-1))</f>
@@ -4347,10 +4420,10 @@
         <v>1</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H69">
         <f>E69*VALUE(LEFT(G69, FIND(":", G69)-1))</f>
@@ -4378,7 +4451,7 @@
         <v>0</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H70">
         <f>E70*VALUE(LEFT(G70, FIND(":", G70)-1))</f>
@@ -4404,7 +4477,7 @@
         <v>1</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="H71">
         <f>E71*VALUE(LEFT(G71, FIND(":", G71)-1))</f>
@@ -4430,7 +4503,7 @@
         <v>1</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H72">
         <f>E72*VALUE(LEFT(G72, FIND(":", G72)-1))</f>
@@ -4456,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H73">
         <f>E73*VALUE(LEFT(G73, FIND(":", G73)-1))</f>
@@ -4482,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H74">
         <f>E74*VALUE(LEFT(G74, FIND(":", G74)-1))</f>
@@ -4508,7 +4581,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H75">
         <f>E75*VALUE(LEFT(G75, FIND(":", G75)-1))</f>
@@ -4538,7 +4611,7 @@
         <v>0</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H76">
         <f>E76*VALUE(LEFT(G76, FIND(":", G76)-1))</f>
@@ -4564,7 +4637,7 @@
         <v>0</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H77">
         <f>E77*VALUE(LEFT(G77, FIND(":", G77)-1))</f>
@@ -4590,7 +4663,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H78">
         <f>E78*VALUE(LEFT(G78, FIND(":", G78)-1))</f>
@@ -4616,7 +4689,7 @@
         <v>0</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H79">
         <f>E79*VALUE(LEFT(G79, FIND(":", G79)-1))</f>
@@ -4642,7 +4715,7 @@
         <v>1</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="H80">
         <f>E80*VALUE(LEFT(G80, FIND(":", G80)-1))</f>
@@ -4668,7 +4741,7 @@
         <v>0</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H81">
         <f>E81*VALUE(LEFT(G81, FIND(":", G81)-1))</f>
@@ -4696,7 +4769,7 @@
         <v>1</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="H82">
         <f>E82*VALUE(LEFT(G82, FIND(":", G82)-1))</f>
@@ -4722,7 +4795,7 @@
         <v>1</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="H83">
         <f>E83*VALUE(LEFT(G83, FIND(":", G83)-1))</f>
@@ -4748,7 +4821,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H84">
         <f>E84*VALUE(LEFT(G84, FIND(":", G84)-1))</f>
@@ -4774,7 +4847,7 @@
         <v>0</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H85">
         <f>E85*VALUE(LEFT(G85, FIND(":", G85)-1))</f>
@@ -4800,7 +4873,7 @@
         <v>0</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H86">
         <f>E86*VALUE(LEFT(G86, FIND(":", G86)-1))</f>
@@ -4826,7 +4899,7 @@
         <v>0</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H87">
         <f>E87*VALUE(LEFT(G87, FIND(":", G87)-1))</f>
@@ -4854,7 +4927,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H88">
         <f>E88*VALUE(LEFT(G88, FIND(":", G88)-1))</f>
@@ -4880,10 +4953,10 @@
         <v>1</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H89">
         <f>E89*VALUE(LEFT(G89, FIND(":", G89)-1))</f>
@@ -4909,7 +4982,7 @@
         <v>1</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H90">
         <f>E90*VALUE(LEFT(G90, FIND(":", G90)-1))</f>
@@ -4935,10 +5008,10 @@
         <v>1</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H91">
         <f>E91*VALUE(LEFT(G91, FIND(":", G91)-1))</f>
@@ -4964,7 +5037,7 @@
         <v>1</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="H92">
         <f>E92*VALUE(LEFT(G92, FIND(":", G92)-1))</f>
@@ -4990,10 +5063,10 @@
         <v>1</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H93">
         <f>E93*VALUE(LEFT(G93, FIND(":", G93)-1))</f>
@@ -5018,10 +5091,13 @@
         <v>270</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>324</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H94">
         <f>E94*VALUE(LEFT(G94, FIND(":", G94)-1))</f>
@@ -5044,10 +5120,13 @@
         <v>271</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>325</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H95">
         <f>E95*VALUE(LEFT(G95, FIND(":", G95)-1))</f>
@@ -5070,10 +5149,13 @@
         <v>272</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>326</v>
       </c>
       <c r="G96" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H96">
         <f>E96*VALUE(LEFT(G96, FIND(":", G96)-1))</f>
@@ -5096,10 +5178,13 @@
         <v>273</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>327</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H97">
         <f>E97*VALUE(LEFT(G97, FIND(":", G97)-1))</f>
@@ -5125,10 +5210,10 @@
         <v>1</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H98">
         <f>E98*VALUE(LEFT(G98, FIND(":", G98)-1))</f>
@@ -5154,7 +5239,7 @@
         <v>1</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H99">
         <f>E99*VALUE(LEFT(G99, FIND(":", G99)-1))</f>
@@ -5177,10 +5262,13 @@
         <v>276</v>
       </c>
       <c r="E100">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>329</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="H100">
         <f>E100*VALUE(LEFT(G100, FIND(":", G100)-1))</f>
@@ -5208,10 +5296,10 @@
         <v>1</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="G101" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H101">
         <f>E101*VALUE(LEFT(G101, FIND(":", G101)-1))</f>
@@ -5237,7 +5325,7 @@
         <v>0</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H102">
         <f>E102*VALUE(LEFT(G102, FIND(":", G102)-1))</f>
@@ -5263,7 +5351,7 @@
         <v>0</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H103">
         <f>E103*VALUE(LEFT(G103, FIND(":", G103)-1))</f>
@@ -5289,7 +5377,7 @@
         <v>0</v>
       </c>
       <c r="G104" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H104">
         <f>E104*VALUE(LEFT(G104, FIND(":", G104)-1))</f>
@@ -5315,7 +5403,7 @@
         <v>0</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H105">
         <f>E105*VALUE(LEFT(G105, FIND(":", G105)-1))</f>
@@ -5341,7 +5429,7 @@
         <v>1</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H106">
         <f>E106*VALUE(LEFT(G106, FIND(":", G106)-1))</f>
@@ -5371,10 +5459,10 @@
         <v>1</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H107">
         <f>E107*VALUE(LEFT(G107, FIND(":", G107)-1))</f>
@@ -5400,10 +5488,10 @@
         <v>1</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="G108" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H108">
         <f>E108*VALUE(LEFT(G108, FIND(":", G108)-1))</f>
@@ -5429,10 +5517,10 @@
         <v>1</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H109">
         <f>E109*VALUE(LEFT(G109, FIND(":", G109)-1))</f>
@@ -5458,10 +5546,10 @@
         <v>1</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="G110" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H110">
         <f>E110*VALUE(LEFT(G110, FIND(":", G110)-1))</f>
@@ -5487,10 +5575,10 @@
         <v>1</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="G111" s="1" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="H111">
         <f>E111*VALUE(LEFT(G111, FIND(":", G111)-1))</f>
@@ -5516,10 +5604,10 @@
         <v>1</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H112">
         <f>E112*VALUE(LEFT(G112, FIND(":", G112)-1))</f>
@@ -5545,7 +5633,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H113">
         <f>E113*VALUE(LEFT(G113, FIND(":", G113)-1))</f>
@@ -5573,10 +5661,10 @@
         <v>1</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H114">
         <f>E114*VALUE(LEFT(G114, FIND(":", G114)-1))</f>
@@ -5602,10 +5690,10 @@
         <v>1</v>
       </c>
       <c r="F115" s="1" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="G115" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H115">
         <f>E115*VALUE(LEFT(G115, FIND(":", G115)-1))</f>
@@ -5631,7 +5719,7 @@
         <v>1</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="H116">
         <f>E116*VALUE(LEFT(G116, FIND(":", G116)-1))</f>
@@ -5657,7 +5745,7 @@
         <v>0</v>
       </c>
       <c r="G117" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H117">
         <f>E117*VALUE(LEFT(G117, FIND(":", G117)-1))</f>
@@ -5683,7 +5771,7 @@
         <v>0</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H118">
         <f>E118*VALUE(LEFT(G118, FIND(":", G118)-1))</f>
@@ -5709,10 +5797,10 @@
         <v>1</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H119">
         <f>E119*VALUE(LEFT(G119, FIND(":", G119)-1))</f>
@@ -5738,7 +5826,7 @@
         <v>0</v>
       </c>
       <c r="G120" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H120">
         <f>E120*VALUE(LEFT(G120, FIND(":", G120)-1))</f>
@@ -5766,7 +5854,7 @@
         <v>0</v>
       </c>
       <c r="G121" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H121">
         <f>E121*VALUE(LEFT(G121, FIND(":", G121)-1))</f>
@@ -5792,7 +5880,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H122">
         <f>E122*VALUE(LEFT(G122, FIND(":", G122)-1))</f>
@@ -5818,7 +5906,7 @@
         <v>0</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H123">
         <f>E123*VALUE(LEFT(G123, FIND(":", G123)-1))</f>
@@ -5844,7 +5932,7 @@
         <v>1</v>
       </c>
       <c r="G124" s="1" t="s">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="H124">
         <f>E124*VALUE(LEFT(G124, FIND(":", G124)-1))</f>
@@ -5870,7 +5958,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H125">
         <f>E125*VALUE(LEFT(G125, FIND(":", G125)-1))</f>
@@ -5896,10 +5984,10 @@
         <v>1</v>
       </c>
       <c r="F126" s="1" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H126">
         <f>E126*VALUE(LEFT(G126, FIND(":", G126)-1))</f>
@@ -5925,10 +6013,10 @@
         <v>1</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H127">
         <f>E127*VALUE(LEFT(G127, FIND(":", G127)-1))</f>
@@ -5954,7 +6042,7 @@
         <v>0</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H128">
         <f>E128*VALUE(LEFT(G128, FIND(":", G128)-1))</f>
@@ -5980,7 +6068,7 @@
         <v>1</v>
       </c>
       <c r="G129" s="1" t="s">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="H129">
         <f>E129*VALUE(LEFT(G129, FIND(":", G129)-1))</f>
@@ -6008,7 +6096,7 @@
         <v>0</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H130">
         <f>E130*VALUE(LEFT(G130, FIND(":", G130)-1))</f>
@@ -6034,10 +6122,10 @@
         <v>1</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G131" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H131">
         <f>E131*VALUE(LEFT(G131, FIND(":", G131)-1))</f>
@@ -6063,10 +6151,10 @@
         <v>1</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="H132">
         <f>E132*VALUE(LEFT(G132, FIND(":", G132)-1))</f>
@@ -6092,7 +6180,7 @@
         <v>0</v>
       </c>
       <c r="G133" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H133">
         <f>E133*VALUE(LEFT(G133, FIND(":", G133)-1))</f>
@@ -6118,7 +6206,7 @@
         <v>1</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="H134">
         <f>E134*VALUE(LEFT(G134, FIND(":", G134)-1))</f>
@@ -6144,7 +6232,7 @@
         <v>0</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H135">
         <f>E135*VALUE(LEFT(G135, FIND(":", G135)-1))</f>
@@ -6170,7 +6258,7 @@
         <v>0</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H136">
         <f>E136*VALUE(LEFT(G136, FIND(":", G136)-1))</f>
@@ -6229,13 +6317,13 @@
       <formula1>"0: None"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: 0 items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G9">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10">
       <formula1>"0: None"</formula1>
@@ -6490,16 +6578,16 @@
       <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G94">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G95">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G96">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G97">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,5: item 1 completed,10: item 2 completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G98">
       <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
@@ -6508,7 +6596,7 @@
       <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G100">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G101">
       <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>

</xml_diff>

<commit_message>
Make clear what version is
so that it points to the specification version and not something more
innate, like a whole version of the framework
</commit_message>
<xml_diff>
--- a/assessments/FinOps Foundation/assessment.xlsx
+++ b/assessments/FinOps Foundation/assessment.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="395">
   <si>
     <t>Sum of Weights</t>
   </si>
@@ -58,21 +58,15 @@
     <t>Anomaly Management</t>
   </si>
   <si>
-    <t>Architecting for Cloud</t>
-  </si>
-  <si>
-    <t>Benchmarking</t>
+    <t>Architecting &amp; Workload Placement</t>
+  </si>
+  <si>
+    <t>Automation, Tools &amp; Services</t>
   </si>
   <si>
     <t>Budgeting</t>
   </si>
   <si>
-    <t>Cloud Policy &amp; Governance</t>
-  </si>
-  <si>
-    <t>Cloud Sustainability</t>
-  </si>
-  <si>
     <t>Data Ingestion</t>
   </si>
   <si>
@@ -85,24 +79,24 @@
     <t>FinOps Practice Operations</t>
   </si>
   <si>
-    <t>FinOps Tools &amp; Services</t>
-  </si>
-  <si>
     <t>Forecasting</t>
   </si>
   <si>
+    <t>Governance, Policy &amp; Risk</t>
+  </si>
+  <si>
     <t>Intersecting Disciplines</t>
   </si>
   <si>
     <t>Invoicing &amp; Chargeback</t>
   </si>
   <si>
+    <t>KPIs &amp; Benchmarking</t>
+  </si>
+  <si>
     <t>Licensing &amp; SaaS</t>
   </si>
   <si>
-    <t>Onboarding Workloads</t>
-  </si>
-  <si>
     <t>Planning &amp; Estimating</t>
   </si>
   <si>
@@ -112,10 +106,13 @@
     <t>Reporting &amp; Analytics</t>
   </si>
   <si>
+    <t>Sustainability</t>
+  </si>
+  <si>
     <t>Unit Economics</t>
   </si>
   <si>
-    <t>Workload Optimization</t>
+    <t>Usage Optimization</t>
   </si>
   <si>
     <t>serial number</t>
@@ -265,6 +262,24 @@
     <t>Resolve Variances &amp; Increase Coverage</t>
   </si>
   <si>
+    <t>Establish Architecture Review Process</t>
+  </si>
+  <si>
+    <t>Assess Workloads for Modernization</t>
+  </si>
+  <si>
+    <t>Estimate Trade-Offs &amp; Document Cases</t>
+  </si>
+  <si>
+    <t>Implement Iteratively &amp; Measure Results</t>
+  </si>
+  <si>
+    <t>Publish Benefits &amp; Update References</t>
+  </si>
+  <si>
+    <t>Strengthen Architecture Collaboration</t>
+  </si>
+  <si>
     <t>Create Workload Selection Criteria</t>
   </si>
   <si>
@@ -283,24 +298,6 @@
     <t>Review Outcomes &amp; Adjust Patterns</t>
   </si>
   <si>
-    <t>Establish Architecture Review Process</t>
-  </si>
-  <si>
-    <t>Assess Workloads for Modernization</t>
-  </si>
-  <si>
-    <t>Estimate Trade-Offs &amp; Document Cases</t>
-  </si>
-  <si>
-    <t>Implement Iteratively &amp; Measure Results</t>
-  </si>
-  <si>
-    <t>Publish Benefits &amp; Update References</t>
-  </si>
-  <si>
-    <t>Strengthen Architecture Collaboration</t>
-  </si>
-  <si>
     <t>Aggregate emissions data by region/service/account with lineage.</t>
   </si>
   <si>
@@ -670,6 +667,24 @@
     <t>112</t>
   </si>
   <si>
+    <t>061</t>
+  </si>
+  <si>
+    <t>062</t>
+  </si>
+  <si>
+    <t>063</t>
+  </si>
+  <si>
+    <t>064</t>
+  </si>
+  <si>
+    <t>065</t>
+  </si>
+  <si>
+    <t>066</t>
+  </si>
+  <si>
     <t>118</t>
   </si>
   <si>
@@ -686,24 +701,6 @@
   </si>
   <si>
     <t>123</t>
-  </si>
-  <si>
-    <t>061</t>
-  </si>
-  <si>
-    <t>062</t>
-  </si>
-  <si>
-    <t>063</t>
-  </si>
-  <si>
-    <t>064</t>
-  </si>
-  <si>
-    <t>065</t>
-  </si>
-  <si>
-    <t>066</t>
   </si>
   <si>
     <t>085</t>
@@ -1021,18 +1018,18 @@
 10*Ceil(x/5)</t>
   </si>
   <si>
-    <t>* Process defined for new accounts and resources deployed
-* Train teams on process
-* Automate process
-10*Ceil(x/3)</t>
-  </si>
-  <si>
     <t>* Define process to address notifications from CSPs
 * Define cadence for review
 * Define exception criteria
 * Define thresholds to change
 * Combine with architecture analysis for SP &amp; RIs
 10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Process defined for new accounts and resources deployed
+* Train teams on process
+* Automate process
+10*Ceil(x/3)</t>
   </si>
   <si>
     <t>* Process for evaluating spot periodically
@@ -1608,9 +1605,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Overview!$A$12:$A$33</c:f>
+              <c:f>Overview!$A$12:$A$32</c:f>
               <c:strCache>
-                <c:ptCount val="22"/>
+                <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>Allocation</c:v>
                 </c:pt>
@@ -1618,74 +1615,71 @@
                   <c:v>Anomaly Management</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Architecting for Cloud</c:v>
+                  <c:v>Architecting &amp; Workload Placement</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Benchmarking</c:v>
+                  <c:v>Automation, Tools &amp; Services</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>Budgeting</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Cloud Policy &amp; Governance</c:v>
+                  <c:v>Data Ingestion</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Cloud Sustainability</c:v>
+                  <c:v>FinOps Assessment</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Data Ingestion</c:v>
+                  <c:v>FinOps Education &amp; Enablement</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>FinOps Assessment</c:v>
+                  <c:v>FinOps Practice Operations</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>FinOps Education &amp; Enablement</c:v>
+                  <c:v>Forecasting</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>FinOps Practice Operations</c:v>
+                  <c:v>Governance, Policy &amp; Risk</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>FinOps Tools &amp; Services</c:v>
+                  <c:v>Intersecting Disciplines</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Forecasting</c:v>
+                  <c:v>Invoicing &amp; Chargeback</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Intersecting Disciplines</c:v>
+                  <c:v>KPIs &amp; Benchmarking</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Invoicing &amp; Chargeback</c:v>
+                  <c:v>Licensing &amp; SaaS</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>Licensing &amp; SaaS</c:v>
+                  <c:v>Planning &amp; Estimating</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Onboarding Workloads</c:v>
+                  <c:v>Rate Optimization</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>Planning &amp; Estimating</c:v>
+                  <c:v>Reporting &amp; Analytics</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>Rate Optimization</c:v>
+                  <c:v>Sustainability</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>Reporting &amp; Analytics</c:v>
+                  <c:v>Unit Economics</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>Unit Economics</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>Workload Optimization</c:v>
+                  <c:v>Usage Optimization</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Overview!$U$12:$U$33</c:f>
+              <c:f>Overview!$U$12:$U$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="22"/>
+                <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1747,9 +1741,6 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1921,7 +1912,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A11:B33" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A11:B32" totalsRowShown="0">
   <tableColumns count="2">
     <tableColumn id="1" name="Capability"/>
     <tableColumn id="2" name="Action Count"/>
@@ -2215,10 +2206,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U34"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
@@ -2268,7 +2259,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="U5">
         <f>SUMIF(Scoring!I2:I136,A5,Scoring!H2:H136)/SUMIF(Scoring!I2:I136,A5,Scoring!E2:E136)</f>
@@ -2280,7 +2271,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="U6">
         <f>SUMIF(Scoring!I2:I136,A6,Scoring!H2:H136)/SUMIF(Scoring!I2:I136,A6,Scoring!E2:E136)</f>
@@ -2354,7 +2345,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="U14">
         <f>SUMIF(Scoring!J2:J136,A14,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A14,Scoring!E2:E136)</f>
@@ -2366,7 +2357,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U15">
         <f>SUMIF(Scoring!J2:J136,A15,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A15,Scoring!E2:E136)</f>
@@ -2390,7 +2381,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U17">
         <f>SUMIF(Scoring!J2:J136,A17,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A17,Scoring!E2:E136)</f>
@@ -2402,7 +2393,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U18">
         <f>SUMIF(Scoring!J2:J136,A18,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A18,Scoring!E2:E136)</f>
@@ -2414,7 +2405,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U19">
         <f>SUMIF(Scoring!J2:J136,A19,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A19,Scoring!E2:E136)</f>
@@ -2426,7 +2417,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U20">
         <f>SUMIF(Scoring!J2:J136,A20,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A20,Scoring!E2:E136)</f>
@@ -2438,7 +2429,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U21">
         <f>SUMIF(Scoring!J2:J136,A21,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A21,Scoring!E2:E136)</f>
@@ -2450,7 +2441,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U22">
         <f>SUMIF(Scoring!J2:J136,A22,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A22,Scoring!E2:E136)</f>
@@ -2462,7 +2453,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U23">
         <f>SUMIF(Scoring!J2:J136,A23,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A23,Scoring!E2:E136)</f>
@@ -2510,7 +2501,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U27">
         <f>SUMIF(Scoring!J2:J136,A27,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A27,Scoring!E2:E136)</f>
@@ -2558,7 +2549,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U31">
         <f>SUMIF(Scoring!J2:J136,A31,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A31,Scoring!E2:E136)</f>
@@ -2577,21 +2568,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:21">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
+    <row r="33" spans="2:2">
       <c r="B33">
-        <v>6</v>
-      </c>
-      <c r="U33">
-        <f>SUMIF(Scoring!J2:J136,A33,Scoring!H2:H136)/SUMIF(Scoring!J2:J136,A33,Scoring!E2:E136)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21">
-      <c r="B34">
-        <f>SUM(Overview!$B$12:$B$33)</f>
+        <f>SUM(Overview!$B$12:$B$32)</f>
         <v>0</v>
       </c>
     </row>
@@ -2612,7 +2591,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="63" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -2620,43 +2599,43 @@
     <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5703125" hidden="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.42578125" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.28515625" hidden="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.42578125" hidden="1" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="D1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -2664,22 +2643,22 @@
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H2">
         <f>E2*VALUE(LEFT(G2, FIND(":", G2)-1))</f>
@@ -2689,26 +2668,26 @@
         <v>6</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H3">
         <f>E3*VALUE(LEFT(G3, FIND(":", G3)-1))</f>
@@ -2718,26 +2697,26 @@
         <v>6</v>
       </c>
       <c r="K3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H4">
         <f>E4*VALUE(LEFT(G4, FIND(":", G4)-1))</f>
@@ -2747,26 +2726,26 @@
         <v>6</v>
       </c>
       <c r="K4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H5">
         <f>E5*VALUE(LEFT(G5, FIND(":", G5)-1))</f>
@@ -2776,26 +2755,26 @@
         <v>6</v>
       </c>
       <c r="K5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F6" s="1">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H6">
         <f>E6*VALUE(LEFT(G6, FIND(":", G6)-1))</f>
@@ -2805,28 +2784,28 @@
         <v>6</v>
       </c>
       <c r="K6" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F7" s="1">
         <v>1</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H7">
         <f>E7*VALUE(LEFT(G7, FIND(":", G7)-1))</f>
@@ -2836,26 +2815,26 @@
         <v>6</v>
       </c>
       <c r="K7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F8" s="1">
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H8">
         <f>E8*VALUE(LEFT(G8, FIND(":", G8)-1))</f>
@@ -2865,26 +2844,26 @@
         <v>6</v>
       </c>
       <c r="K8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F9" s="1">
         <v>1</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H9">
         <f>E9*VALUE(LEFT(G9, FIND(":", G9)-1))</f>
@@ -2894,26 +2873,26 @@
         <v>6</v>
       </c>
       <c r="K9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H10">
         <f>E10*VALUE(LEFT(G10, FIND(":", G10)-1))</f>
@@ -2923,26 +2902,26 @@
         <v>6</v>
       </c>
       <c r="K10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H11">
         <f>E11*VALUE(LEFT(G11, FIND(":", G11)-1))</f>
@@ -2952,28 +2931,28 @@
         <v>6</v>
       </c>
       <c r="K11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E12" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F12" s="1">
         <v>0</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H12">
         <f>E12*VALUE(LEFT(G12, FIND(":", G12)-1))</f>
@@ -2983,26 +2962,26 @@
         <v>6</v>
       </c>
       <c r="K12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E13" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F13" s="1">
         <v>0</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H13">
         <f>E13*VALUE(LEFT(G13, FIND(":", G13)-1))</f>
@@ -3012,26 +2991,26 @@
         <v>6</v>
       </c>
       <c r="K13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H14">
         <f>E14*VALUE(LEFT(G14, FIND(":", G14)-1))</f>
@@ -3041,26 +3020,26 @@
         <v>6</v>
       </c>
       <c r="K14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H15">
         <f>E15*VALUE(LEFT(G15, FIND(":", G15)-1))</f>
@@ -3070,26 +3049,26 @@
         <v>6</v>
       </c>
       <c r="K15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H16">
         <f>E16*VALUE(LEFT(G16, FIND(":", G16)-1))</f>
@@ -3099,28 +3078,28 @@
         <v>6</v>
       </c>
       <c r="K16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H17">
         <f>E17*VALUE(LEFT(G17, FIND(":", G17)-1))</f>
@@ -3130,26 +3109,26 @@
         <v>6</v>
       </c>
       <c r="K17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E18" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H18">
         <f>E18*VALUE(LEFT(G18, FIND(":", G18)-1))</f>
@@ -3159,26 +3138,26 @@
         <v>6</v>
       </c>
       <c r="K18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E19" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H19">
         <f>E19*VALUE(LEFT(G19, FIND(":", G19)-1))</f>
@@ -3188,26 +3167,26 @@
         <v>6</v>
       </c>
       <c r="K19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E20" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H20">
         <f>E20*VALUE(LEFT(G20, FIND(":", G20)-1))</f>
@@ -3217,26 +3196,26 @@
         <v>6</v>
       </c>
       <c r="K20" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H21">
         <f>E21*VALUE(LEFT(G21, FIND(":", G21)-1))</f>
@@ -3246,26 +3225,26 @@
         <v>6</v>
       </c>
       <c r="K21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H22">
         <f>E22*VALUE(LEFT(G22, FIND(":", G22)-1))</f>
@@ -3275,28 +3254,28 @@
         <v>6</v>
       </c>
       <c r="K22" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E23" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H23">
         <f>E23*VALUE(LEFT(G23, FIND(":", G23)-1))</f>
@@ -3306,26 +3285,26 @@
         <v>6</v>
       </c>
       <c r="K23" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E24" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F24" s="1">
         <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H24">
         <f>E24*VALUE(LEFT(G24, FIND(":", G24)-1))</f>
@@ -3335,26 +3314,26 @@
         <v>6</v>
       </c>
       <c r="K24" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E25" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H25">
         <f>E25*VALUE(LEFT(G25, FIND(":", G25)-1))</f>
@@ -3364,26 +3343,26 @@
         <v>6</v>
       </c>
       <c r="K25" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F26" s="1">
         <v>1</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H26">
         <f>E26*VALUE(LEFT(G26, FIND(":", G26)-1))</f>
@@ -3393,26 +3372,26 @@
         <v>6</v>
       </c>
       <c r="K26" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E27" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H27">
         <f>E27*VALUE(LEFT(G27, FIND(":", G27)-1))</f>
@@ -3422,28 +3401,28 @@
         <v>6</v>
       </c>
       <c r="K27" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F28" s="1">
         <v>0</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H28">
         <f>E28*VALUE(LEFT(G28, FIND(":", G28)-1))</f>
@@ -3453,26 +3432,26 @@
         <v>6</v>
       </c>
       <c r="K28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E29" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F29" s="1">
         <v>0</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H29">
         <f>E29*VALUE(LEFT(G29, FIND(":", G29)-1))</f>
@@ -3482,26 +3461,26 @@
         <v>6</v>
       </c>
       <c r="K29" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E30" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F30" s="1">
         <v>0</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H30">
         <f>E30*VALUE(LEFT(G30, FIND(":", G30)-1))</f>
@@ -3511,26 +3490,26 @@
         <v>6</v>
       </c>
       <c r="K30" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E31" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H31">
         <f>E31*VALUE(LEFT(G31, FIND(":", G31)-1))</f>
@@ -3540,26 +3519,26 @@
         <v>6</v>
       </c>
       <c r="K31" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E32" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H32">
         <f>E32*VALUE(LEFT(G32, FIND(":", G32)-1))</f>
@@ -3569,26 +3548,26 @@
         <v>6</v>
       </c>
       <c r="K32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H33">
         <f>E33*VALUE(LEFT(G33, FIND(":", G33)-1))</f>
@@ -3598,28 +3577,28 @@
         <v>6</v>
       </c>
       <c r="K33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H34">
         <f>E34*VALUE(LEFT(G34, FIND(":", G34)-1))</f>
@@ -3629,26 +3608,26 @@
         <v>6</v>
       </c>
       <c r="K34" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E35" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F35" s="1">
         <v>0</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H35">
         <f>E35*VALUE(LEFT(G35, FIND(":", G35)-1))</f>
@@ -3658,26 +3637,26 @@
         <v>6</v>
       </c>
       <c r="K35" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E36" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H36">
         <f>E36*VALUE(LEFT(G36, FIND(":", G36)-1))</f>
@@ -3687,26 +3666,26 @@
         <v>6</v>
       </c>
       <c r="K36" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E37" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F37" s="1">
         <v>0</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H37">
         <f>E37*VALUE(LEFT(G37, FIND(":", G37)-1))</f>
@@ -3716,26 +3695,26 @@
         <v>6</v>
       </c>
       <c r="K37" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E38" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F38" s="1">
         <v>0</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H38">
         <f>E38*VALUE(LEFT(G38, FIND(":", G38)-1))</f>
@@ -3745,26 +3724,26 @@
         <v>6</v>
       </c>
       <c r="K38" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E39" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F39" s="1">
         <v>1</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H39">
         <f>E39*VALUE(LEFT(G39, FIND(":", G39)-1))</f>
@@ -3774,206 +3753,204 @@
         <v>6</v>
       </c>
       <c r="K39" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="2"/>
+      <c r="A40" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="B40" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E40" t="s">
         <v>314</v>
       </c>
       <c r="F40" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H40">
         <f>E40*VALUE(LEFT(G40, FIND(":", G40)-1))</f>
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K40" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E41" t="s">
         <v>314</v>
       </c>
       <c r="F41" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="H41">
         <f>E41*VALUE(LEFT(G41, FIND(":", G41)-1))</f>
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K41" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E42" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F42" s="1">
         <v>1</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="H42">
         <f>E42*VALUE(LEFT(G42, FIND(":", G42)-1))</f>
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K42" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E43" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F43" s="1">
         <v>0</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H43">
         <f>E43*VALUE(LEFT(G43, FIND(":", G43)-1))</f>
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K43" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E44" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F44" s="1">
         <v>0</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H44">
         <f>E44*VALUE(LEFT(G44, FIND(":", G44)-1))</f>
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K44" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E45" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F45" s="1">
         <v>0</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H45">
         <f>E45*VALUE(LEFT(G45, FIND(":", G45)-1))</f>
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K45" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
       <c r="C46" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E46" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="F46" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="H46">
         <f>E46*VALUE(LEFT(G46, FIND(":", G46)-1))</f>
@@ -3990,19 +3967,19 @@
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E47" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="F47" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="H47">
         <f>E47*VALUE(LEFT(G47, FIND(":", G47)-1))</f>
@@ -4019,19 +3996,19 @@
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E48" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F48" s="1">
         <v>1</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="H48">
         <f>E48*VALUE(LEFT(G48, FIND(":", G48)-1))</f>
@@ -4048,19 +4025,19 @@
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E49" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F49" s="1">
         <v>0</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H49">
         <f>E49*VALUE(LEFT(G49, FIND(":", G49)-1))</f>
@@ -4077,19 +4054,19 @@
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E50" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F50" s="1">
         <v>0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H50">
         <f>E50*VALUE(LEFT(G50, FIND(":", G50)-1))</f>
@@ -4106,19 +4083,19 @@
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E51" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F51" s="1">
         <v>0</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H51">
         <f>E51*VALUE(LEFT(G51, FIND(":", G51)-1))</f>
@@ -4134,22 +4111,22 @@
     <row r="52" spans="1:11">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E52" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F52" s="1">
         <v>0</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H52">
         <f>E52*VALUE(LEFT(G52, FIND(":", G52)-1))</f>
@@ -4159,26 +4136,26 @@
         <v>7</v>
       </c>
       <c r="K52" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:11">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E53" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F53" s="1">
         <v>0</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H53">
         <f>E53*VALUE(LEFT(G53, FIND(":", G53)-1))</f>
@@ -4188,26 +4165,26 @@
         <v>7</v>
       </c>
       <c r="K53" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:11">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E54" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F54" s="1">
         <v>0</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H54">
         <f>E54*VALUE(LEFT(G54, FIND(":", G54)-1))</f>
@@ -4217,26 +4194,26 @@
         <v>7</v>
       </c>
       <c r="K54" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="55" spans="1:11">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E55" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F55" s="1">
         <v>0</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H55">
         <f>E55*VALUE(LEFT(G55, FIND(":", G55)-1))</f>
@@ -4246,26 +4223,26 @@
         <v>7</v>
       </c>
       <c r="K55" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="56" spans="1:11">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E56" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F56" s="1">
         <v>0</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H56">
         <f>E56*VALUE(LEFT(G56, FIND(":", G56)-1))</f>
@@ -4275,26 +4252,26 @@
         <v>7</v>
       </c>
       <c r="K56" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="57" spans="1:11">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E57" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F57" s="1">
         <v>0</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H57">
         <f>E57*VALUE(LEFT(G57, FIND(":", G57)-1))</f>
@@ -4304,28 +4281,28 @@
         <v>7</v>
       </c>
       <c r="K57" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58" spans="1:11">
       <c r="A58" s="2"/>
       <c r="B58" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E58" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F58" s="1">
         <v>1</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H58">
         <f>E58*VALUE(LEFT(G58, FIND(":", G58)-1))</f>
@@ -4335,26 +4312,26 @@
         <v>7</v>
       </c>
       <c r="K58" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:11">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E59" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F59" s="1">
         <v>0</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H59">
         <f>E59*VALUE(LEFT(G59, FIND(":", G59)-1))</f>
@@ -4364,26 +4341,26 @@
         <v>7</v>
       </c>
       <c r="K59" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:11">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E60" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F60" s="1">
         <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H60">
         <f>E60*VALUE(LEFT(G60, FIND(":", G60)-1))</f>
@@ -4393,26 +4370,26 @@
         <v>7</v>
       </c>
       <c r="K60" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="61" spans="1:11">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E61" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F61" s="1">
         <v>1</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H61">
         <f>E61*VALUE(LEFT(G61, FIND(":", G61)-1))</f>
@@ -4422,26 +4399,26 @@
         <v>7</v>
       </c>
       <c r="K61" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62" spans="1:11">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E62" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F62" s="1">
         <v>0</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H62">
         <f>E62*VALUE(LEFT(G62, FIND(":", G62)-1))</f>
@@ -4451,26 +4428,26 @@
         <v>7</v>
       </c>
       <c r="K62" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:11">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E63" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F63" s="1">
         <v>0</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H63">
         <f>E63*VALUE(LEFT(G63, FIND(":", G63)-1))</f>
@@ -4480,28 +4457,28 @@
         <v>7</v>
       </c>
       <c r="K63" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="64" spans="1:11">
       <c r="A64" s="2"/>
       <c r="B64" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E64" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F64" s="1">
         <v>1</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H64">
         <f>E64*VALUE(LEFT(G64, FIND(":", G64)-1))</f>
@@ -4511,26 +4488,26 @@
         <v>7</v>
       </c>
       <c r="K64" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="65" spans="1:11">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E65" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F65" s="1">
         <v>1</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H65">
         <f>E65*VALUE(LEFT(G65, FIND(":", G65)-1))</f>
@@ -4540,26 +4517,26 @@
         <v>7</v>
       </c>
       <c r="K65" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="66" spans="1:11">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E66" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F66" s="1">
         <v>0</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H66">
         <f>E66*VALUE(LEFT(G66, FIND(":", G66)-1))</f>
@@ -4569,26 +4546,26 @@
         <v>7</v>
       </c>
       <c r="K66" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67" spans="1:11">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E67" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F67" s="1">
         <v>0</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H67">
         <f>E67*VALUE(LEFT(G67, FIND(":", G67)-1))</f>
@@ -4598,26 +4575,26 @@
         <v>7</v>
       </c>
       <c r="K67" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="68" spans="1:11">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E68" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F68" s="1">
         <v>0</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H68">
         <f>E68*VALUE(LEFT(G68, FIND(":", G68)-1))</f>
@@ -4627,26 +4604,26 @@
         <v>7</v>
       </c>
       <c r="K68" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69" spans="1:11">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E69" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F69" s="1">
         <v>1</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H69">
         <f>E69*VALUE(LEFT(G69, FIND(":", G69)-1))</f>
@@ -4656,28 +4633,28 @@
         <v>7</v>
       </c>
       <c r="K69" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="70" spans="1:11">
       <c r="A70" s="2"/>
       <c r="B70" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E70" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F70" s="1">
         <v>0</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H70">
         <f>E70*VALUE(LEFT(G70, FIND(":", G70)-1))</f>
@@ -4687,26 +4664,26 @@
         <v>7</v>
       </c>
       <c r="K70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="71" spans="1:11">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E71" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F71" s="1">
         <v>1</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H71">
         <f>E71*VALUE(LEFT(G71, FIND(":", G71)-1))</f>
@@ -4716,26 +4693,26 @@
         <v>7</v>
       </c>
       <c r="K71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="72" spans="1:11">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E72" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F72" s="1">
         <v>1</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H72">
         <f>E72*VALUE(LEFT(G72, FIND(":", G72)-1))</f>
@@ -4745,26 +4722,26 @@
         <v>7</v>
       </c>
       <c r="K72" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="73" spans="1:11">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E73" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F73" s="1">
         <v>0</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H73">
         <f>E73*VALUE(LEFT(G73, FIND(":", G73)-1))</f>
@@ -4774,26 +4751,26 @@
         <v>7</v>
       </c>
       <c r="K73" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:11">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E74" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F74" s="1">
         <v>0</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H74">
         <f>E74*VALUE(LEFT(G74, FIND(":", G74)-1))</f>
@@ -4803,26 +4780,26 @@
         <v>7</v>
       </c>
       <c r="K74" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75" spans="1:11">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E75" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F75" s="1">
         <v>0</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H75">
         <f>E75*VALUE(LEFT(G75, FIND(":", G75)-1))</f>
@@ -4832,7 +4809,7 @@
         <v>7</v>
       </c>
       <c r="K75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -4840,22 +4817,22 @@
         <v>8</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E76" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F76" s="1">
         <v>0</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H76">
         <f>E76*VALUE(LEFT(G76, FIND(":", G76)-1))</f>
@@ -4865,26 +4842,26 @@
         <v>8</v>
       </c>
       <c r="K76" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:11">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E77" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F77" s="1">
         <v>0</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H77">
         <f>E77*VALUE(LEFT(G77, FIND(":", G77)-1))</f>
@@ -4894,26 +4871,26 @@
         <v>8</v>
       </c>
       <c r="K77" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="78" spans="1:11">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E78" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F78" s="1">
         <v>0</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H78">
         <f>E78*VALUE(LEFT(G78, FIND(":", G78)-1))</f>
@@ -4923,26 +4900,26 @@
         <v>8</v>
       </c>
       <c r="K78" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="79" spans="1:11">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E79" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F79" s="1">
         <v>0</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H79">
         <f>E79*VALUE(LEFT(G79, FIND(":", G79)-1))</f>
@@ -4952,26 +4929,26 @@
         <v>8</v>
       </c>
       <c r="K79" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="80" spans="1:11">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E80" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F80" s="1">
         <v>1</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="H80">
         <f>E80*VALUE(LEFT(G80, FIND(":", G80)-1))</f>
@@ -4981,26 +4958,26 @@
         <v>8</v>
       </c>
       <c r="K80" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="81" spans="1:11">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E81" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F81" s="1">
         <v>0</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H81">
         <f>E81*VALUE(LEFT(G81, FIND(":", G81)-1))</f>
@@ -5010,7 +4987,7 @@
         <v>8</v>
       </c>
       <c r="K81" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -5019,19 +4996,19 @@
         <v>15</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E82" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F82" s="1">
         <v>1</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H82">
         <f>E82*VALUE(LEFT(G82, FIND(":", G82)-1))</f>
@@ -5048,19 +5025,19 @@
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E83" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F83" s="1">
         <v>1</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H83">
         <f>E83*VALUE(LEFT(G83, FIND(":", G83)-1))</f>
@@ -5077,19 +5054,19 @@
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E84" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F84" s="1">
         <v>0</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H84">
         <f>E84*VALUE(LEFT(G84, FIND(":", G84)-1))</f>
@@ -5106,19 +5083,19 @@
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E85" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F85" s="1">
         <v>0</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H85">
         <f>E85*VALUE(LEFT(G85, FIND(":", G85)-1))</f>
@@ -5135,19 +5112,19 @@
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E86" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F86" s="1">
         <v>0</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H86">
         <f>E86*VALUE(LEFT(G86, FIND(":", G86)-1))</f>
@@ -5164,19 +5141,19 @@
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E87" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F87" s="1">
         <v>0</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H87">
         <f>E87*VALUE(LEFT(G87, FIND(":", G87)-1))</f>
@@ -5192,22 +5169,22 @@
     <row r="88" spans="1:11">
       <c r="A88" s="2"/>
       <c r="B88" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E88" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F88" s="1">
         <v>0</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H88">
         <f>E88*VALUE(LEFT(G88, FIND(":", G88)-1))</f>
@@ -5217,26 +5194,26 @@
         <v>8</v>
       </c>
       <c r="K88" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="89" spans="1:11">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E89" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F89" s="1">
         <v>1</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H89">
         <f>E89*VALUE(LEFT(G89, FIND(":", G89)-1))</f>
@@ -5246,26 +5223,26 @@
         <v>8</v>
       </c>
       <c r="K89" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="90" spans="1:11">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E90" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F90" s="1">
         <v>1</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H90">
         <f>E90*VALUE(LEFT(G90, FIND(":", G90)-1))</f>
@@ -5275,26 +5252,26 @@
         <v>8</v>
       </c>
       <c r="K90" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="91" spans="1:11">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E91" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F91" s="1">
         <v>1</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H91">
         <f>E91*VALUE(LEFT(G91, FIND(":", G91)-1))</f>
@@ -5304,26 +5281,26 @@
         <v>8</v>
       </c>
       <c r="K91" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92" spans="1:11">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E92" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F92" s="1">
         <v>1</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H92">
         <f>E92*VALUE(LEFT(G92, FIND(":", G92)-1))</f>
@@ -5333,26 +5310,26 @@
         <v>8</v>
       </c>
       <c r="K92" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93" spans="1:11">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E93" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F93" s="1">
         <v>1</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H93">
         <f>E93*VALUE(LEFT(G93, FIND(":", G93)-1))</f>
@@ -5362,28 +5339,28 @@
         <v>8</v>
       </c>
       <c r="K93" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="94" spans="1:11">
       <c r="A94" s="2"/>
       <c r="B94" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E94" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F94" s="1">
         <v>1</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H94">
         <f>E94*VALUE(LEFT(G94, FIND(":", G94)-1))</f>
@@ -5393,26 +5370,26 @@
         <v>8</v>
       </c>
       <c r="K94" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="95" spans="1:11">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E95" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F95" s="1">
         <v>1</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H95">
         <f>E95*VALUE(LEFT(G95, FIND(":", G95)-1))</f>
@@ -5422,26 +5399,26 @@
         <v>8</v>
       </c>
       <c r="K95" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="96" spans="1:11">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E96" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F96" s="1">
         <v>1</v>
       </c>
       <c r="G96" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H96">
         <f>E96*VALUE(LEFT(G96, FIND(":", G96)-1))</f>
@@ -5451,26 +5428,26 @@
         <v>8</v>
       </c>
       <c r="K96" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="97" spans="1:11">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E97" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F97" s="1">
         <v>1</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H97">
         <f>E97*VALUE(LEFT(G97, FIND(":", G97)-1))</f>
@@ -5480,26 +5457,26 @@
         <v>8</v>
       </c>
       <c r="K97" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="98" spans="1:11">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E98" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F98" s="1">
         <v>1</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H98">
         <f>E98*VALUE(LEFT(G98, FIND(":", G98)-1))</f>
@@ -5509,26 +5486,26 @@
         <v>8</v>
       </c>
       <c r="K98" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99" spans="1:11">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E99" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F99" s="1">
         <v>1</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H99">
         <f>E99*VALUE(LEFT(G99, FIND(":", G99)-1))</f>
@@ -5538,26 +5515,26 @@
         <v>8</v>
       </c>
       <c r="K99" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="100" spans="1:11">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E100" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F100" s="1">
         <v>1</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H100">
         <f>E100*VALUE(LEFT(G100, FIND(":", G100)-1))</f>
@@ -5567,28 +5544,28 @@
         <v>8</v>
       </c>
       <c r="K100" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="101" spans="1:11">
       <c r="A101" s="2"/>
       <c r="B101" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E101" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F101" s="1">
         <v>1</v>
       </c>
       <c r="G101" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H101">
         <f>E101*VALUE(LEFT(G101, FIND(":", G101)-1))</f>
@@ -5598,26 +5575,26 @@
         <v>8</v>
       </c>
       <c r="K101" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102" spans="1:11">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E102" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F102" s="1">
         <v>0</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H102">
         <f>E102*VALUE(LEFT(G102, FIND(":", G102)-1))</f>
@@ -5627,26 +5604,26 @@
         <v>8</v>
       </c>
       <c r="K102" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="103" spans="1:11">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E103" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F103" s="1">
         <v>0</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H103">
         <f>E103*VALUE(LEFT(G103, FIND(":", G103)-1))</f>
@@ -5656,26 +5633,26 @@
         <v>8</v>
       </c>
       <c r="K103" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104" spans="1:11">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E104" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F104" s="1">
         <v>0</v>
       </c>
       <c r="G104" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H104">
         <f>E104*VALUE(LEFT(G104, FIND(":", G104)-1))</f>
@@ -5685,26 +5662,26 @@
         <v>8</v>
       </c>
       <c r="K104" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="105" spans="1:11">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E105" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F105" s="1">
         <v>0</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H105">
         <f>E105*VALUE(LEFT(G105, FIND(":", G105)-1))</f>
@@ -5714,26 +5691,26 @@
         <v>8</v>
       </c>
       <c r="K105" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106" spans="1:11">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E106" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F106" s="1">
         <v>1</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H106">
         <f>E106*VALUE(LEFT(G106, FIND(":", G106)-1))</f>
@@ -5743,7 +5720,7 @@
         <v>8</v>
       </c>
       <c r="K106" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -5754,19 +5731,19 @@
         <v>11</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E107" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F107" s="1">
         <v>1</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H107">
         <f>E107*VALUE(LEFT(G107, FIND(":", G107)-1))</f>
@@ -5783,19 +5760,19 @@
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E108" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F108" s="1">
         <v>1</v>
       </c>
       <c r="G108" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H108">
         <f>E108*VALUE(LEFT(G108, FIND(":", G108)-1))</f>
@@ -5812,19 +5789,19 @@
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E109" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F109" s="1">
         <v>1</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H109">
         <f>E109*VALUE(LEFT(G109, FIND(":", G109)-1))</f>
@@ -5841,19 +5818,19 @@
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E110" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F110" s="1">
         <v>1</v>
       </c>
       <c r="G110" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H110">
         <f>E110*VALUE(LEFT(G110, FIND(":", G110)-1))</f>
@@ -5870,19 +5847,19 @@
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E111" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F111" s="1">
         <v>1</v>
       </c>
       <c r="G111" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H111">
         <f>E111*VALUE(LEFT(G111, FIND(":", G111)-1))</f>
@@ -5899,19 +5876,19 @@
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E112" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F112" s="1">
         <v>1</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H112">
         <f>E112*VALUE(LEFT(G112, FIND(":", G112)-1))</f>
@@ -5928,19 +5905,19 @@
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E113" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F113" s="1">
         <v>0</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H113">
         <f>E113*VALUE(LEFT(G113, FIND(":", G113)-1))</f>
@@ -5959,19 +5936,19 @@
         <v>12</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E114" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F114" s="1">
         <v>1</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H114">
         <f>E114*VALUE(LEFT(G114, FIND(":", G114)-1))</f>
@@ -5988,19 +5965,19 @@
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E115" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F115" s="1">
         <v>1</v>
       </c>
       <c r="G115" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H115">
         <f>E115*VALUE(LEFT(G115, FIND(":", G115)-1))</f>
@@ -6017,19 +5994,19 @@
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E116" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F116" s="1">
         <v>1</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H116">
         <f>E116*VALUE(LEFT(G116, FIND(":", G116)-1))</f>
@@ -6046,19 +6023,19 @@
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E117" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F117" s="1">
         <v>0</v>
       </c>
       <c r="G117" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H117">
         <f>E117*VALUE(LEFT(G117, FIND(":", G117)-1))</f>
@@ -6075,19 +6052,19 @@
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E118" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F118" s="1">
         <v>0</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H118">
         <f>E118*VALUE(LEFT(G118, FIND(":", G118)-1))</f>
@@ -6104,19 +6081,19 @@
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E119" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F119" s="1">
         <v>1</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H119">
         <f>E119*VALUE(LEFT(G119, FIND(":", G119)-1))</f>
@@ -6133,19 +6110,19 @@
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E120" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F120" s="1">
         <v>0</v>
       </c>
       <c r="G120" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H120">
         <f>E120*VALUE(LEFT(G120, FIND(":", G120)-1))</f>
@@ -6161,22 +6138,22 @@
     <row r="121" spans="1:11">
       <c r="A121" s="2"/>
       <c r="B121" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E121" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F121" s="1">
         <v>0</v>
       </c>
       <c r="G121" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H121">
         <f>E121*VALUE(LEFT(G121, FIND(":", G121)-1))</f>
@@ -6186,26 +6163,26 @@
         <v>9</v>
       </c>
       <c r="K121" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="122" spans="1:11">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E122" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F122" s="1">
         <v>0</v>
       </c>
       <c r="G122" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H122">
         <f>E122*VALUE(LEFT(G122, FIND(":", G122)-1))</f>
@@ -6215,26 +6192,26 @@
         <v>9</v>
       </c>
       <c r="K122" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="123" spans="1:11">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E123" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F123" s="1">
         <v>0</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H123">
         <f>E123*VALUE(LEFT(G123, FIND(":", G123)-1))</f>
@@ -6244,26 +6221,26 @@
         <v>9</v>
       </c>
       <c r="K123" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="124" spans="1:11">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E124" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F124" s="1">
         <v>1</v>
       </c>
       <c r="G124" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="H124">
         <f>E124*VALUE(LEFT(G124, FIND(":", G124)-1))</f>
@@ -6273,26 +6250,26 @@
         <v>9</v>
       </c>
       <c r="K124" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="125" spans="1:11">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E125" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F125" s="1">
         <v>0</v>
       </c>
       <c r="G125" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H125">
         <f>E125*VALUE(LEFT(G125, FIND(":", G125)-1))</f>
@@ -6302,26 +6279,26 @@
         <v>9</v>
       </c>
       <c r="K125" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="126" spans="1:11">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E126" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F126" s="1">
         <v>1</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H126">
         <f>E126*VALUE(LEFT(G126, FIND(":", G126)-1))</f>
@@ -6331,26 +6308,26 @@
         <v>9</v>
       </c>
       <c r="K126" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="127" spans="1:11">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E127" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F127" s="1">
         <v>1</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H127">
         <f>E127*VALUE(LEFT(G127, FIND(":", G127)-1))</f>
@@ -6360,26 +6337,26 @@
         <v>9</v>
       </c>
       <c r="K127" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="128" spans="1:11">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E128" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F128" s="1">
         <v>0</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H128">
         <f>E128*VALUE(LEFT(G128, FIND(":", G128)-1))</f>
@@ -6389,26 +6366,26 @@
         <v>9</v>
       </c>
       <c r="K128" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="129" spans="1:11">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E129" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F129" s="1">
         <v>1</v>
       </c>
       <c r="G129" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="H129">
         <f>E129*VALUE(LEFT(G129, FIND(":", G129)-1))</f>
@@ -6418,28 +6395,28 @@
         <v>9</v>
       </c>
       <c r="K129" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="130" spans="1:11">
       <c r="A130" s="2"/>
       <c r="B130" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E130" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F130" s="1">
         <v>0</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H130">
         <f>E130*VALUE(LEFT(G130, FIND(":", G130)-1))</f>
@@ -6449,26 +6426,26 @@
         <v>9</v>
       </c>
       <c r="K130" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="131" spans="1:11">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E131" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F131" s="1">
         <v>1</v>
       </c>
       <c r="G131" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H131">
         <f>E131*VALUE(LEFT(G131, FIND(":", G131)-1))</f>
@@ -6478,26 +6455,26 @@
         <v>9</v>
       </c>
       <c r="K131" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132" spans="1:11">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E132" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F132" s="1">
         <v>1</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H132">
         <f>E132*VALUE(LEFT(G132, FIND(":", G132)-1))</f>
@@ -6507,26 +6484,26 @@
         <v>9</v>
       </c>
       <c r="K132" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="133" spans="1:11">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E133" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F133" s="1">
         <v>0</v>
       </c>
       <c r="G133" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H133">
         <f>E133*VALUE(LEFT(G133, FIND(":", G133)-1))</f>
@@ -6536,26 +6513,26 @@
         <v>9</v>
       </c>
       <c r="K133" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="134" spans="1:11">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E134" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F134" s="1">
         <v>1</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="H134">
         <f>E134*VALUE(LEFT(G134, FIND(":", G134)-1))</f>
@@ -6565,26 +6542,26 @@
         <v>9</v>
       </c>
       <c r="K134" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="135" spans="1:11">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E135" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F135" s="1">
         <v>0</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H135">
         <f>E135*VALUE(LEFT(G135, FIND(":", G135)-1))</f>
@@ -6594,26 +6571,26 @@
         <v>9</v>
       </c>
       <c r="K135" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="136" spans="1:11">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E136" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F136" s="1">
         <v>0</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H136">
         <f>E136*VALUE(LEFT(G136, FIND(":", G136)-1))</f>
@@ -6623,13 +6600,13 @@
         <v>9</v>
       </c>
       <c r="K136" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A2:A45"/>
-    <mergeCell ref="A46:A75"/>
+  <mergeCells count="25">
+    <mergeCell ref="A2:A39"/>
+    <mergeCell ref="A40:A75"/>
     <mergeCell ref="A76:A106"/>
     <mergeCell ref="A107:A136"/>
     <mergeCell ref="B2:B6"/>
@@ -6639,8 +6616,7 @@
     <mergeCell ref="B23:B27"/>
     <mergeCell ref="B28:B33"/>
     <mergeCell ref="B34:B39"/>
-    <mergeCell ref="B40:B45"/>
-    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="B40:B51"/>
     <mergeCell ref="B52:B57"/>
     <mergeCell ref="B58:B63"/>
     <mergeCell ref="B64:B69"/>
@@ -6771,31 +6747,31 @@
       <formula1>"0: Not done,10: Defined"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G40">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: Does not exist,10: Exists"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G41">
-      <formula1>"0: None"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G42">
+      <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G43">
+      <formula1>"0: None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G44">
+      <formula1>"0: None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G45">
+      <formula1>"0: None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G46">
+      <formula1>"0: None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G47">
+      <formula1>"0: None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G48">
       <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G43">
-      <formula1>"0: None"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G44">
-      <formula1>"0: None"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G45">
-      <formula1>"0: None"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G46">
-      <formula1>"0: Does not exist,10: Exists"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G47">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G48">
-      <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G49">
       <formula1>"0: None"</formula1>

</xml_diff>

<commit_message>
Update UI view some more
to clean up the UX
</commit_message>
<xml_diff>
--- a/assessments/FinOps Foundation/assessment.xlsx
+++ b/assessments/FinOps Foundation/assessment.xlsx
@@ -1556,11 +1556,12 @@
         <c:axId val="50020002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="10"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="cross"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
@@ -1757,11 +1758,12 @@
         <c:axId val="50030002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="10"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="cross"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50030001"/>
         <c:crosses val="autoZero"/>
@@ -2298,6 +2300,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:21"/>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Update specifications where need be
to include fixes for action 135 that was missing a Title
</commit_message>
<xml_diff>
--- a/assessments/FinOps Foundation/assessment.xlsx
+++ b/assessments/FinOps Foundation/assessment.xlsx
@@ -544,7 +544,7 @@
     <t>Optimize Pipelines for Timeliness</t>
   </si>
   <si>
-    <t>Define ingestion frequency; include mandatory metadata.</t>
+    <t>Define Data Ingestion Requirements</t>
   </si>
   <si>
     <t>Gather Requirements &amp; Define KPIs</t>
@@ -997,7 +997,7 @@
     <t>2.1.0</t>
   </si>
   <si>
-    <t>1.6.0</t>
+    <t>1.6.1</t>
   </si>
   <si>
     <t>* Select which teams or groups are in scope for the planned assessments
@@ -2801,7 +2801,7 @@
   <cols>
     <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>

</xml_diff>